<commit_message>
feat(projections): add Cash Flow (unrealized/prepaid) + Balance Sheet (deferred/accrued rev) to each Year P&L; fix cohort renewal cash
Each Year (monthly) sheet now carries all three statements: P&L (accrual) -> Cash Flow
(prepaid/unrealized cash basis) -> Balance Sheet (Cash = Deferred Revenue + Retained
Earnings), 5-yr full monthly detail. Fixes the revenue/cash model to a cohort/annual-
renewal basis so renewal cash is collected and deferred (unearned) revenue stays a
positive liability. Balance sheet reconciles to $0.00. Adds deferred + cumulative cash
to the 5-Year Summary and Exec Dashboard.

Co-authored-by: marcellmiller27 <marcellmiller27@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/JHI_5yr_Consolidated_Projections.xlsx
+++ b/public/downloads/JHI_5yr_Consolidated_Projections.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,6 +127,7 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -495,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -543,7 +544,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4,271</t>
+          <t>4,591</t>
         </is>
       </c>
     </row>
@@ -555,7 +556,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>$19,330,428</t>
+          <t>$20,778,610</t>
         </is>
       </c>
     </row>
@@ -579,7 +580,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>$18,074,289</t>
+          <t>$19,410,475</t>
         </is>
       </c>
     </row>
@@ -591,7 +592,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>$15,424,578</t>
+          <t>$16,704,738</t>
         </is>
       </c>
     </row>
@@ -603,7 +604,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>85.3%</t>
+          <t>86.1%</t>
         </is>
       </c>
     </row>
@@ -615,7 +616,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>$54,095,505</t>
+          <t>$57,932,294</t>
         </is>
       </c>
     </row>
@@ -627,7 +628,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>$43,434,925</t>
+          <t>$47,059,361</t>
         </is>
       </c>
     </row>
@@ -639,24 +640,48 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>$27,802,675</t>
+          <t>$67,605,711</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Ending cash (Yr 5)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>$56,732,777</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Ending deferred (unearned) revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>$9,673,416</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Headcount at Yr 5</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>6 staged hires</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Audited-realistic basis: conservative rep ramp, 85% annual renewal, accrual revenue, commission expensed upfront, EBITDA-gated hiring. Working model — see Assumptions to tweak.</t>
         </is>
@@ -686,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -775,19 +800,19 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1034</v>
+        <v>1102</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>2050</v>
+        <v>2197</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>2913</v>
+        <v>3128</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>3647</v>
+        <v>3918</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>4271</v>
+        <v>4591</v>
       </c>
     </row>
     <row r="8">
@@ -797,19 +822,19 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>2313617</v>
+        <v>2415902</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>7231859</v>
+        <v>7717025</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>11446603</v>
+        <v>12262584</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>15029136</v>
+        <v>16126309</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>18074289</v>
+        <v>19410475</v>
       </c>
     </row>
     <row r="9">
@@ -822,16 +847,16 @@
         <v>4990224</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>5703113</v>
+        <v>9944803</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>5703113</v>
+        <v>14156195</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>5703113</v>
+        <v>17735879</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>5703113</v>
+        <v>20778610</v>
       </c>
     </row>
     <row r="10">
@@ -841,19 +866,19 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>2216906</v>
+        <v>2315510</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>6946624</v>
+        <v>7411447</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>10984643</v>
+        <v>11766409</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>14416960</v>
+        <v>15468127</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>17334429</v>
+        <v>18614588</v>
       </c>
     </row>
     <row r="11">
@@ -885,10 +910,10 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>101667</v>
+        <v>130417</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>553333</v>
+        <v>576667</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>680000</v>
@@ -907,41 +932,85 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>1234705</v>
+        <v>1304559</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>5193739</v>
+        <v>5635228</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>9074793</v>
+        <v>9856559</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>12507110</v>
+        <v>13558277</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>15424578</v>
+        <v>16704738</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Deferred (unearned) revenue (end)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>2574322</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>4802100</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>6695712</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>8305282</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>9673416</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>3878880</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>11741887</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>23492058</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>38659905</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>56732777</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n">
-        <v>0.5336686636289441</v>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>0.7181748037433172</v>
-      </c>
-      <c r="D14" s="19" t="n">
-        <v>0.7927935503838175</v>
-      </c>
-      <c r="E14" s="19" t="n">
-        <v>0.8321908356478666</v>
-      </c>
-      <c r="F14" s="19" t="n">
-        <v>0.8533988799476074</v>
+      <c r="B16" s="19" t="n">
+        <v>0.5399882515237564</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>0.7302332716297044</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0.8037914010196672</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>0.8407551513982537</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>0.8606042489228986</v>
       </c>
     </row>
   </sheetData>
@@ -982,35 +1051,35 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Internal planning model consolidating prior JHI forecasts from user-supplied assumptions — illustrative only, not a forecast, guarantee, or offer.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Sales headcount (qualified 1099 reps) is the key unknown variable; the Sales Scaling tab shows output at each attainable headcount toward the 100/mo (1,200/yr) goal.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Staged staffing is EBITDA-gated so salaries are added only when the business supports them.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Founder signature of provenance: JHI-SIG: 69M2705M</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>© 2026 JHI Research &amp; Analytics Firm, Inc.. All rights reserved. Confidential.</t>
         </is>
@@ -1704,7 +1773,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Mo 7</t>
+          <t>Mo 6</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1791,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Mo 9</t>
+          <t>Mo 8</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1809,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Mo 11</t>
+          <t>Mo 10</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1827,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Mo 15</t>
+          <t>Mo 14</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1845,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Mo 19</t>
+          <t>Mo 18</t>
         </is>
       </c>
     </row>
@@ -1811,10 +1880,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -1840,7 +1909,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 1 — monthly consolidated P&amp;L</t>
+          <t>Year 1 — monthly P&amp;L, Cash Flow &amp; Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -1979,86 +2048,86 @@
         <v>26</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>559</v>
+        <v>578</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>657</v>
+        <v>682</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>753</v>
+        <v>788</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>848</v>
+        <v>892</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>942</v>
+        <v>998</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>1034</v>
+        <v>1102</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>1034</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Recognized revenue</t>
+          <t>Recognized revenue (accrual)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
         <v>9901</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>29571</v>
+        <v>29704</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>58876</v>
+        <v>59407</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>97689</v>
+        <v>99012</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>135980</v>
+        <v>138617</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>173756</v>
+        <v>178222</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>211024</v>
+        <v>217827</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>247790</v>
+        <v>257432</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>284062</v>
+        <v>297037</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>319845</v>
+        <v>336642</v>
       </c>
       <c r="L8" s="17" t="n">
-        <v>355148</v>
+        <v>376247</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>389975</v>
+        <v>415852</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>2313617</v>
+        <v>2415902</v>
       </c>
     </row>
     <row r="9">
@@ -2071,40 +2140,40 @@
         <v>1836</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>2505</v>
+        <v>2509</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>3500</v>
+        <v>3518</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>4819</v>
+        <v>4864</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>6120</v>
+        <v>6210</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>7404</v>
+        <v>7555</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>8670</v>
+        <v>8901</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>9919</v>
+        <v>10247</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>11151</v>
+        <v>11592</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>12367</v>
+        <v>12938</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>13567</v>
+        <v>14284</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>14852</v>
+        <v>15937</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>96711</v>
+        <v>100392</v>
       </c>
     </row>
     <row r="10">
@@ -2117,40 +2186,40 @@
         <v>8065</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>27066</v>
+        <v>27194</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>55376</v>
+        <v>55889</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>92870</v>
+        <v>94148</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>129860</v>
+        <v>132408</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>166352</v>
+        <v>170667</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>202354</v>
+        <v>208926</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>237871</v>
+        <v>247185</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>272910</v>
+        <v>285445</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>307478</v>
+        <v>323704</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>341581</v>
+        <v>361963</v>
       </c>
       <c r="M10" s="17" t="n">
-        <v>375123</v>
+        <v>399915</v>
       </c>
       <c r="N10" s="17" t="n">
-        <v>2216906</v>
+        <v>2315510</v>
       </c>
     </row>
     <row r="11">
@@ -2316,25 +2385,25 @@
         <v>4583</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>4583</v>
+        <v>10833</v>
       </c>
       <c r="I14" s="12" t="n">
         <v>10833</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>10833</v>
+        <v>18750</v>
       </c>
       <c r="K14" s="12" t="n">
         <v>18750</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>18750</v>
+        <v>33333</v>
       </c>
       <c r="M14" s="12" t="n">
         <v>33333</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>101667</v>
+        <v>130417</v>
       </c>
     </row>
     <row r="15">
@@ -2389,44 +2458,44 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="18" t="n">
         <v>-20757</v>
       </c>
-      <c r="C16" s="17" t="n">
-        <v>-19579</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>-9091</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>10581</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>47571</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>79480</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>115481</v>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>144748</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>179788</v>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>206439</v>
-      </c>
-      <c r="L16" s="17" t="n">
-        <v>240542</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>259501</v>
+      <c r="C16" s="18" t="n">
+        <v>-19450</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>-8578</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>11859</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>50119</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>83795</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>115804</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>154063</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>184406</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>222665</v>
+      </c>
+      <c r="L16" s="18" t="n">
+        <v>246341</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>284293</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>1234705</v>
+        <v>1304559</v>
       </c>
     </row>
     <row r="17">
@@ -2439,40 +2508,448 @@
         <v>-2.096453646156183</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>-0.6621028878690988</v>
+        <v>-0.6548023991389401</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>-0.1544037457521031</v>
+        <v>-0.1443895873846295</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.108315087359281</v>
+        <v>0.1197755373170947</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>0.3498381454394333</v>
+        <v>0.3615605907606907</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0.4574230463881475</v>
+        <v>0.4701686704612729</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>0.5472438359507733</v>
+        <v>0.5316315790339492</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>0.5841580062967661</v>
+        <v>0.5984610629317541</v>
       </c>
       <c r="J17" s="19" t="n">
-        <v>0.6329182078685021</v>
+        <v>0.6208172393153437</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.645433902539695</v>
+        <v>0.6614297081452658</v>
       </c>
       <c r="L17" s="19" t="n">
-        <v>0.677301134572094</v>
+        <v>0.6547321871404388</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>0.6654297487272941</v>
+        <v>0.6836395067820309</v>
       </c>
       <c r="N17" s="19" t="n">
-        <v>0.5336686636289441</v>
+        <v>0.5399882515237564</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>CASH FLOW — based on prepaid (unrealized) revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bookings — prepaid cash in</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>118815</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>237630</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>356445</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>475259</v>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>4990224</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total cash outflows</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>30659</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>49154</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>67985</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>87153</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>88499</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>94428</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>102023</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>103369</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>112631</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>113977</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>129906</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>131559</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>1111343</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>88156</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>188476</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>288459</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>388106</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>386761</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>380832</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>373236</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>371890</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>362628</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>361282</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>345353</v>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>343700</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>3878880</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>88156</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>276632</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>565091</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>953198</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>1339958</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>1720790</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>2094026</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>2465916</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>2828544</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>3189827</v>
+      </c>
+      <c r="L23" s="18" t="n">
+        <v>3535180</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>3878880</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>3878880</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET — period end (Cash = Deferred Rev + Retained Earnings)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Assets: Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>88156</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>276632</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>565091</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>953198</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>1339958</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>1720790</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>2094026</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>2465916</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>2828544</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>3189827</v>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>3535180</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>3878880</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>3878880</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities: Deferred (unearned/accrued) revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>108914</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>316840</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>613877</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>990124</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>1326766</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>1623803</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>1881235</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>2099062</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>2277285</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>2415902</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>2514914</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>2574322</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>2574322</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity: Retained earnings</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>-20757</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>-40208</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>-48785</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>-36926</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>13192</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>96987</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>212791</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>366854</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>551260</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>773925</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>1020266</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>1304559</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>1304559</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Balance check (Assets − Liab − Equity)</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2499,10 +2976,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -2528,7 +3005,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 2 — monthly consolidated P&amp;L</t>
+          <t>Year 2 — monthly P&amp;L, Cash Flow &amp; Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -2664,89 +3141,89 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1125</v>
+        <v>1204</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1215</v>
+        <v>1301</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>1304</v>
+        <v>1394</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>1391</v>
+        <v>1483</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>1477</v>
+        <v>1572</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>1562</v>
+        <v>1662</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>1646</v>
+        <v>1751</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>1729</v>
+        <v>1840</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>1811</v>
+        <v>1929</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>1892</v>
+        <v>2019</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>1971</v>
+        <v>2108</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>2050</v>
+        <v>2197</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>2050</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Recognized revenue</t>
+          <t>Recognized revenue (accrual)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>424334</v>
+        <v>453972</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>458231</v>
+        <v>490606</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>491672</v>
+        <v>525756</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>524663</v>
+        <v>559420</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>557210</v>
+        <v>593084</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>589320</v>
+        <v>626748</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>620997</v>
+        <v>660413</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>652248</v>
+        <v>694077</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>683079</v>
+        <v>727741</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>713495</v>
+        <v>761405</v>
       </c>
       <c r="L8" s="17" t="n">
-        <v>743503</v>
+        <v>795069</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>773106</v>
+        <v>828734</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>7231859</v>
+        <v>7717025</v>
       </c>
     </row>
     <row r="9">
@@ -2756,43 +3233,43 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>16292</v>
+        <v>17535</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>17714</v>
+        <v>19071</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>19116</v>
+        <v>20545</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>20499</v>
+        <v>21957</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>21864</v>
+        <v>23368</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>23210</v>
+        <v>24780</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>24539</v>
+        <v>26191</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>25849</v>
+        <v>27603</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>27142</v>
+        <v>29014</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>28417</v>
+        <v>30426</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>29675</v>
+        <v>31838</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>30917</v>
+        <v>33249</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>285234</v>
+        <v>305577</v>
       </c>
     </row>
     <row r="10">
@@ -2802,43 +3279,43 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>408042</v>
+        <v>436437</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>440517</v>
+        <v>471535</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>472556</v>
+        <v>505211</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>504164</v>
+        <v>537463</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>535346</v>
+        <v>569716</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>566109</v>
+        <v>601969</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>596458</v>
+        <v>634221</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>626399</v>
+        <v>666474</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>655938</v>
+        <v>698727</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>685078</v>
+        <v>730979</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>713827</v>
+        <v>763232</v>
       </c>
       <c r="M10" s="17" t="n">
-        <v>742189</v>
+        <v>795485</v>
       </c>
       <c r="N10" s="17" t="n">
-        <v>6946624</v>
+        <v>7411447</v>
       </c>
     </row>
     <row r="11">
@@ -2992,7 +3469,7 @@
         <v>33333</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>33333</v>
+        <v>42500</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>42500</v>
@@ -3004,7 +3481,7 @@
         <v>42500</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>42500</v>
+        <v>56667</v>
       </c>
       <c r="I14" s="12" t="n">
         <v>56667</v>
@@ -3022,7 +3499,7 @@
         <v>56667</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>553333</v>
+        <v>576667</v>
       </c>
     </row>
     <row r="15">
@@ -3077,44 +3554,44 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
-        <v>287370</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>314796</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>341785</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>359176</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>390359</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>421122</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>451471</v>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>467245</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>496783</v>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>525924</v>
-      </c>
-      <c r="L16" s="17" t="n">
-        <v>554673</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>583035</v>
+      <c r="B16" s="18" t="n">
+        <v>315765</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>345813</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>365273</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>392476</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>424728</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>456981</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>475067</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>507320</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>539572</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>571825</v>
+      </c>
+      <c r="L16" s="18" t="n">
+        <v>604078</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>636330</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>5193739</v>
+        <v>5635228</v>
       </c>
     </row>
     <row r="17">
@@ -3124,43 +3601,451 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>0.6772251452065911</v>
+        <v>0.6955600332893153</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>0.6869802829905435</v>
+        <v>0.7048695321255009</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.6951479818058919</v>
+        <v>0.6947574850603522</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.6845845392610146</v>
+        <v>0.7015762715977953</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>0.7005590837567575</v>
+        <v>0.7161351625016059</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0.7145896847940153</v>
+        <v>0.7291300651250701</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>0.7270097547530119</v>
+        <v>0.7193489119896387</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>0.7163608404835545</v>
+        <v>0.7309273797186825</v>
       </c>
       <c r="J17" s="19" t="n">
-        <v>0.7272704240842538</v>
+        <v>0.7414346422700735</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.7371093609190283</v>
+        <v>0.7510127840756976</v>
       </c>
       <c r="L17" s="19" t="n">
-        <v>0.746027106485783</v>
+        <v>0.7597798254544446</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>0.7541465366087703</v>
+        <v>0.7678346101859337</v>
       </c>
       <c r="N17" s="19" t="n">
-        <v>0.7181748037433172</v>
+        <v>0.7302332716297044</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>CASH FLOW — based on prepaid (unrealized) revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bookings — prepaid cash in</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>576252</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>677245</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>778237</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>879230</v>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>9944803</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total cash outflows</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>138207</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>144793</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>160483</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>166944</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>168356</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>169767</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>185345</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>186757</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>188169</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>189580</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>190992</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>192403</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>2081796</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>438045</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>532452</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>617754</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>712286</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>710874</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>709463</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>693884</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>692473</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>691061</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>689650</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>688238</v>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>686827</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>7863006</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>4316925</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>4849377</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>5467131</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>6179417</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>6890291</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>7599754</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>8293638</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>8986111</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>9677172</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>10366822</v>
+      </c>
+      <c r="L23" s="18" t="n">
+        <v>11055060</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>11741887</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>11741887</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET — period end (Cash = Deferred Rev + Retained Earnings)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Assets: Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>4316925</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>4849377</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>5467131</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>6179417</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>6890291</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>7599754</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>8293638</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>8986111</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>9677172</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>10366822</v>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>11055060</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>11741887</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>11741887</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities: Deferred (unearned/accrued) revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>2696602</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>2883240</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>3135722</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>3455532</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>3741678</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>3994159</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>4212977</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>4398130</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>4549619</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>4667443</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>4751604</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>4802100</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>4802100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity: Retained earnings</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>1620323</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>1966137</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>2331409</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>2723885</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>3148614</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>3605595</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>4080662</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>4587981</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>5127554</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>5699379</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>6303456</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>6939787</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>6939787</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Balance check (Assets − Liab − Equity)</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3187,10 +4072,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -3216,7 +4101,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 3 — monthly consolidated P&amp;L</t>
+          <t>Year 3 — monthly P&amp;L, Cash Flow &amp; Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -3352,89 +4237,89 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>2127</v>
+        <v>2283</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>2203</v>
+        <v>2366</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>2279</v>
+        <v>2445</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>2353</v>
+        <v>2521</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>2427</v>
+        <v>2597</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>2499</v>
+        <v>2672</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>2570</v>
+        <v>2748</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2641</v>
+        <v>2824</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>2710</v>
+        <v>2900</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2779</v>
+        <v>2976</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>2846</v>
+        <v>3052</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>2913</v>
+        <v>3128</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>2913</v>
+        <v>3128</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Recognized revenue</t>
+          <t>Recognized revenue (accrual)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>802311</v>
+        <v>861135</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>831123</v>
+        <v>892275</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>859548</v>
+        <v>922152</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>887590</v>
+        <v>950766</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>915256</v>
+        <v>979381</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>942549</v>
+        <v>1007995</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>969474</v>
+        <v>1036610</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>996038</v>
+        <v>1065225</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>1022244</v>
+        <v>1093839</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>1048098</v>
+        <v>1122454</v>
       </c>
       <c r="L8" s="17" t="n">
-        <v>1073604</v>
+        <v>1151068</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>1098767</v>
+        <v>1179683</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>11446603</v>
+        <v>12262584</v>
       </c>
     </row>
     <row r="9">
@@ -3444,43 +4329,43 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>32141</v>
+        <v>34608</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>33349</v>
+        <v>35913</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>34541</v>
+        <v>37166</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>35717</v>
+        <v>38366</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>36877</v>
+        <v>39566</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>38021</v>
+        <v>40766</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>39150</v>
+        <v>41965</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>40264</v>
+        <v>43165</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>41363</v>
+        <v>44365</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>42447</v>
+        <v>45565</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>43517</v>
+        <v>46765</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>44572</v>
+        <v>47964</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>461960</v>
+        <v>496174</v>
       </c>
     </row>
     <row r="10">
@@ -3490,43 +4375,43 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>770170</v>
+        <v>826528</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>797774</v>
+        <v>856361</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>825007</v>
+        <v>884986</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>851874</v>
+        <v>912400</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>878379</v>
+        <v>939815</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>904527</v>
+        <v>967230</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>930324</v>
+        <v>994645</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>955774</v>
+        <v>1022059</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>980881</v>
+        <v>1049474</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>1005651</v>
+        <v>1076889</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>1030088</v>
+        <v>1104304</v>
       </c>
       <c r="M10" s="17" t="n">
-        <v>1054195</v>
+        <v>1131718</v>
       </c>
       <c r="N10" s="17" t="n">
-        <v>10984643</v>
+        <v>11766409</v>
       </c>
     </row>
     <row r="11">
@@ -3765,44 +4650,44 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
-        <v>611016</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>638620</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>665853</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>692719</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>719224</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>745373</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>771170</v>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>796620</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>821727</v>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>846497</v>
-      </c>
-      <c r="L16" s="17" t="n">
-        <v>870933</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>895041</v>
+      <c r="B16" s="18" t="n">
+        <v>667374</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>697207</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>725831</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>753246</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>780661</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>808076</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>835490</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>862905</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>890320</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>917735</v>
+      </c>
+      <c r="L16" s="18" t="n">
+        <v>945150</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>972564</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>9074793</v>
+        <v>9856559</v>
       </c>
     </row>
     <row r="17">
@@ -3812,43 +4697,451 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>0.7615696047254535</v>
+        <v>0.7749925537130929</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>0.7683816132365259</v>
+        <v>0.7813817405025653</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.7746544794986617</v>
+        <v>0.7871062891324042</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.7804492621109229</v>
+        <v>0.792251659397361</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>0.7858181358416789</v>
+        <v>0.7970963650499594</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0.7908059506579019</v>
+        <v>0.801666011533833</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>0.7954514735727323</v>
+        <v>0.8059833770427145</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>0.7997883861273273</v>
+        <v>0.8100687922551669</v>
       </c>
       <c r="J17" s="19" t="n">
-        <v>0.8038460918250864</v>
+        <v>0.8139404604666873</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.8076503744622451</v>
+        <v>0.8176147287552809</v>
       </c>
       <c r="L17" s="19" t="n">
-        <v>0.8112239385186985</v>
+        <v>0.821106318701368</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>0.8145868555447341</v>
+        <v>0.8244285235294194</v>
       </c>
       <c r="N17" s="19" t="n">
-        <v>0.7927935503838175</v>
+        <v>0.8037914010196672</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>CASH FLOW — based on prepaid (unrealized) revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bookings — prepaid cash in</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>965074</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>1050917</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>1136761</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>1222605</v>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>14156195</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total cash outflows</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>193762</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>195068</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>196320</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>197520</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>198720</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>199920</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>201120</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>202319</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>203519</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>204719</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>205919</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>207119</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>2406024</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>771312</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>855850</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>940441</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>1025085</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>1023885</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>1022685</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>1021485</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>1020285</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>1019086</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>1017886</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>1016686</v>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>1015486</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>11750171</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>12513199</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>13369048</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>14309489</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>15334574</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>16358459</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>17381144</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>18402629</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>19422914</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>20442000</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>21459886</v>
+      </c>
+      <c r="L23" s="18" t="n">
+        <v>22476572</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>23492058</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>23492058</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET — period end (Cash = Deferred Rev + Retained Earnings)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Assets: Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>12513199</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>13369048</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>14309489</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>15334574</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>16358459</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>17381144</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>18402629</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>19422914</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>20442000</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>21459886</v>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>22476572</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>23492058</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>23492058</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities: Deferred (unearned/accrued) revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>4906038</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>5064681</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>5279290</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>5551129</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>5794353</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>6008962</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>6194957</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>6352337</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>6481103</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>6581254</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>6652790</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>6695712</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>6695712</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity: Retained earnings</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>7607160</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>8304367</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>9030199</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>9783445</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>10564106</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>11372182</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>12207672</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>13070577</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>13960897</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>14878632</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>15823782</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>16796346</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>16796346</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Balance check (Assets − Liab − Equity)</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3875,10 +5168,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -3904,7 +5197,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 4 — monthly consolidated P&amp;L</t>
+          <t>Year 4 — monthly P&amp;L, Cash Flow &amp; Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -4040,89 +5333,89 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>2979</v>
+        <v>3201</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>3044</v>
+        <v>3271</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>3108</v>
+        <v>3338</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>3171</v>
+        <v>3403</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3233</v>
+        <v>3467</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3295</v>
+        <v>3532</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>3356</v>
+        <v>3596</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>3415</v>
+        <v>3660</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3474</v>
+        <v>3725</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>3533</v>
+        <v>3789</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3590</v>
+        <v>3854</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>3647</v>
+        <v>3918</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>3647</v>
+        <v>3918</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Recognized revenue</t>
+          <t>Recognized revenue (accrual)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>1123591</v>
+        <v>1207224</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1148082</v>
+        <v>1233693</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>1172243</v>
+        <v>1259088</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>1196079</v>
+        <v>1283411</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>1219594</v>
+        <v>1307733</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>1242793</v>
+        <v>1332056</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>1265680</v>
+        <v>1356378</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>1288259</v>
+        <v>1380700</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>1310535</v>
+        <v>1405023</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>1332510</v>
+        <v>1429345</v>
       </c>
       <c r="L8" s="17" t="n">
-        <v>1354190</v>
+        <v>1453668</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>1375579</v>
+        <v>1477990</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>15029136</v>
+        <v>16126309</v>
       </c>
     </row>
     <row r="9">
@@ -4132,43 +5425,43 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>45613</v>
+        <v>49119</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>46639</v>
+        <v>50229</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>47653</v>
+        <v>51294</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>48652</v>
+        <v>52314</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>49638</v>
+        <v>53334</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>50611</v>
+        <v>54354</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>51570</v>
+        <v>55373</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>52517</v>
+        <v>56393</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>53451</v>
+        <v>57413</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>54373</v>
+        <v>58433</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>55282</v>
+        <v>59453</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>56178</v>
+        <v>60473</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>612177</v>
+        <v>658181</v>
       </c>
     </row>
     <row r="10">
@@ -4178,43 +5471,43 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>1077979</v>
+        <v>1158105</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>1101442</v>
+        <v>1183464</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>1124590</v>
+        <v>1207794</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>1147427</v>
+        <v>1231097</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>1169956</v>
+        <v>1254399</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>1192183</v>
+        <v>1277702</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>1214110</v>
+        <v>1301005</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>1235742</v>
+        <v>1324307</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>1257084</v>
+        <v>1347610</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>1278138</v>
+        <v>1370912</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>1298909</v>
+        <v>1394215</v>
       </c>
       <c r="M10" s="17" t="n">
-        <v>1319400</v>
+        <v>1417517</v>
       </c>
       <c r="N10" s="17" t="n">
-        <v>14416960</v>
+        <v>15468127</v>
       </c>
     </row>
     <row r="11">
@@ -4453,44 +5746,44 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
-        <v>918825</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>942288</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>965436</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>988273</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>1010802</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>1033028</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>1054956</v>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>1076588</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>1097929</v>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>1118984</v>
-      </c>
-      <c r="L16" s="17" t="n">
-        <v>1139755</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>1160246</v>
+      <c r="B16" s="18" t="n">
+        <v>998951</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>1024310</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>1048640</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>1071943</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>1095245</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>1118548</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>1141850</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>1165153</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>1188455</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>1211758</v>
+      </c>
+      <c r="L16" s="18" t="n">
+        <v>1235061</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>1258363</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>12507110</v>
+        <v>13558277</v>
       </c>
     </row>
     <row r="17">
@@ -4500,43 +5793,451 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>0.8177569350841115</v>
+        <v>0.8274774028262871</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>0.8207500346093296</v>
+        <v>0.8302792177280547</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.8235803198560417</v>
+        <v>0.8328567130185759</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.8262604845769389</v>
+        <v>0.8352296698945683</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>0.8288019369081303</v>
+        <v>0.8375143580263418</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0.8312149581199043</v>
+        <v>0.8397156125879174</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>0.8335088384108823</v>
+        <v>0.8418379219385134</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>0.8356919935273989</v>
+        <v>0.8438854581699585</v>
       </c>
       <c r="J17" s="19" t="n">
-        <v>0.8377720652943119</v>
+        <v>0.8458621044812636</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.8397560085885066</v>
+        <v>0.8477714797582818</v>
       </c>
       <c r="L17" s="19" t="n">
-        <v>0.8416501668412226</v>
+        <v>0.8496169606858063</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>0.8434603377963612</v>
+        <v>0.8514017016763566</v>
       </c>
       <c r="N17" s="19" t="n">
-        <v>0.8321908356478666</v>
+        <v>0.8407551513982537</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>CASH FLOW — based on prepaid (unrealized) revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bookings — prepaid cash in</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>1295572</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>1368539</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>1441506</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>1514473</v>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>17735879</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total cash outflows</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>208274</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>209383</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>210448</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>211468</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>212488</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>213508</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>214528</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>215547</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>216567</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>217587</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>218607</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>219627</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>2568032</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>1087298</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>1159156</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>1231058</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>1303005</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>1301986</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>1300966</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>1299946</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>1298926</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>1297906</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>1296886</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>1295867</v>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>1294847</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>15167847</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>24579356</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>25738512</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>26969570</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>28272576</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>29574561</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>30875527</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>32175473</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>33474399</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>34772305</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>36069192</v>
+      </c>
+      <c r="L23" s="18" t="n">
+        <v>37365058</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>38659905</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>38659905</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET — period end (Cash = Deferred Rev + Retained Earnings)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Assets: Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>24579356</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>25738512</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>26969570</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>28272576</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>29574561</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>30875527</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>32175473</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>33474399</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>34772305</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>36069192</v>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>37365058</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>38659905</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>38659905</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities: Deferred (unearned/accrued) revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>6784059</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>6918906</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>7101323</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>7332386</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>7539126</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>7721544</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>7879640</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>8013413</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>8122864</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>8207992</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>8268798</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>8305282</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>8305282</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity: Retained earnings</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>17795297</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>18819607</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>19868247</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>20940190</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>22035435</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>23153983</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>24295833</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>25460986</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>26649442</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>27861200</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>29096260</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>30354623</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>30354623</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Balance check (Assets − Liab − Equity)</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4563,10 +6264,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -4592,7 +6293,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 5 — monthly consolidated P&amp;L</t>
+          <t>Year 5 — monthly P&amp;L, Cash Flow &amp; Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -4728,89 +6429,89 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>3703</v>
+        <v>3980</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>3758</v>
+        <v>4040</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>3812</v>
+        <v>4097</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>3866</v>
+        <v>4152</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3919</v>
+        <v>4207</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3971</v>
+        <v>4262</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>4023</v>
+        <v>4317</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>4074</v>
+        <v>4371</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>4124</v>
+        <v>4426</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>4174</v>
+        <v>4481</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>4223</v>
+        <v>4536</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>4271</v>
+        <v>4591</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>4271</v>
+        <v>4591</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Recognized revenue</t>
+          <t>Recognized revenue (accrual)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>1396680</v>
+        <v>1501400</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1417497</v>
+        <v>1523898</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>1438033</v>
+        <v>1545485</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>1458294</v>
+        <v>1566159</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>1478282</v>
+        <v>1586833</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>1498001</v>
+        <v>1607507</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>1517455</v>
+        <v>1628181</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>1536647</v>
+        <v>1648855</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>1555581</v>
+        <v>1669529</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>1574261</v>
+        <v>1690203</v>
       </c>
       <c r="L8" s="17" t="n">
-        <v>1592689</v>
+        <v>1710877</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>1610869</v>
+        <v>1731551</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>18074289</v>
+        <v>19410475</v>
       </c>
     </row>
     <row r="9">
@@ -4820,43 +6521,43 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>57063</v>
+        <v>61454</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>57936</v>
+        <v>62398</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>58797</v>
+        <v>63303</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>59647</v>
+        <v>64170</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>60485</v>
+        <v>65036</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>61312</v>
+        <v>65903</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>62127</v>
+        <v>66770</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>62932</v>
+        <v>67637</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>63726</v>
+        <v>68504</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>64509</v>
+        <v>69371</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>65282</v>
+        <v>70238</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>66044</v>
+        <v>71104</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>739861</v>
+        <v>795888</v>
       </c>
     </row>
     <row r="10">
@@ -4866,43 +6567,43 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>1339616</v>
+        <v>1439946</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>1359560</v>
+        <v>1461501</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>1379236</v>
+        <v>1482182</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>1398647</v>
+        <v>1501989</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>1417797</v>
+        <v>1521796</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>1436690</v>
+        <v>1541603</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>1455328</v>
+        <v>1561411</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>1473715</v>
+        <v>1581218</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>1491855</v>
+        <v>1601025</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>1509752</v>
+        <v>1620832</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>1527407</v>
+        <v>1640639</v>
       </c>
       <c r="M10" s="17" t="n">
-        <v>1544825</v>
+        <v>1660446</v>
       </c>
       <c r="N10" s="17" t="n">
-        <v>17334429</v>
+        <v>18614588</v>
       </c>
     </row>
     <row r="11">
@@ -5141,44 +6842,44 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
-        <v>1180462</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>1200406</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>1220082</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>1239493</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>1258643</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>1277535</v>
-      </c>
-      <c r="H16" s="17" t="n">
-        <v>1296174</v>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>1314561</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>1332701</v>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>1350597</v>
-      </c>
-      <c r="L16" s="17" t="n">
-        <v>1368253</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>1385671</v>
+      <c r="B16" s="18" t="n">
+        <v>1280792</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>1302347</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>1323028</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>1342835</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>1362642</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>1382449</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>1402256</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>1422063</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>1441871</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>1461678</v>
+      </c>
+      <c r="L16" s="18" t="n">
+        <v>1481485</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>1501292</v>
       </c>
       <c r="N16" s="18" t="n">
-        <v>15424578</v>
+        <v>16704738</v>
       </c>
     </row>
     <row r="17">
@@ -5188,43 +6889,451 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>0.8451918309609903</v>
+        <v>0.8530649019621432</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>0.8468495179473224</v>
+        <v>0.8546151493048237</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.8484378767115808</v>
+        <v>0.8560601213036356</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.8499610305358732</v>
+        <v>0.8574066954811294</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>0.8514227824677338</v>
+        <v>0.8587181820042</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0.8528266458230757</v>
+        <v>0.8599959346525303</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>0.854175871267701</v>
+        <v>0.8612412384466425</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>0.8554734709168913</v>
+        <v>0.8624553139585542</v>
       </c>
       <c r="J17" s="19" t="n">
-        <v>0.8567222398292309</v>
+        <v>0.8636393213021584</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.8579247752175536</v>
+        <v>0.8647943638307457</v>
       </c>
       <c r="L17" s="19" t="n">
-        <v>0.8590834936549648</v>
+        <v>0.8659214915664483</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>0.860200646515883</v>
+        <v>0.8670217043840029</v>
       </c>
       <c r="N17" s="19" t="n">
-        <v>0.8533988799476074</v>
+        <v>0.8606042489228986</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>CASH FLOW — based on prepaid (unrealized) revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bookings — prepaid cash in</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>1576496</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>1638518</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>1700540</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>1762562</v>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>20778610</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total cash outflows</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>220608</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>221552</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>222457</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>223324</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>224191</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>225057</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>225924</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>226791</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>227658</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>228525</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>229392</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>230259</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>2705738</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>1355887</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>1416966</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>1478083</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>1539238</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>1538371</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>1537504</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>1536638</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>1535771</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>1534904</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>1534037</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>1533170</v>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>1532303</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>18072872</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative cash (end)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>40015792</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>41432758</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>42910841</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>44450079</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>45988450</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>47525955</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>49062592</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>50598363</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>52133267</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>53667304</v>
+      </c>
+      <c r="L23" s="18" t="n">
+        <v>55200474</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>56732777</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>56732777</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET — period end (Cash = Deferred Rev + Retained Earnings)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Assets: Cash</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>40015792</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>41432758</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>42910841</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>44450079</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>45988450</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>47525955</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>49062592</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>50598363</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>52133267</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>53667304</v>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>55200474</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>56732777</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>56732777</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities: Deferred (unearned/accrued) revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>8380377</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>8494996</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>8650052</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>8846455</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>9022184</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>9177239</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>9311621</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>9425328</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>9518361</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>9590720</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>9642405</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>9673416</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>9673416</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity: Retained earnings</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>31635415</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>32937762</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>34260789</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>35603624</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>36966266</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>38348715</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>39750972</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>41173035</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>42614906</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>44076584</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>45558069</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>47059361</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>47059361</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Balance check (Assets − Liab − Equity)</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>